<commit_message>
refactor: Make use of `amdt_idx` in attribution instead of num amdt and lecture
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/mappings_attributions_for_tests.xlsx
+++ b/tests/integration/test_data/mappings_attributions_for_tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204FC208-8424-CC45-8F6D-FC0A17E4012A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{096F565F-BAF3-7B4C-9A53-CB843C0AF657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{5BF04301-CB7D-4341-BBF7-1B79619915A7}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{5BF04301-CB7D-4341-BBF7-1B79619915A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Code et Article" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
tests: Update integration tests for newest features
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/mappings_attributions_for_tests.xlsx
+++ b/tests/integration/test_data/mappings_attributions_for_tests.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF11C3D1-8888-E745-B592-BB227C76785B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0676A3-88E4-404B-AD70-DD89B63BDB71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="500" windowWidth="19200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="500" windowWidth="19200" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Code et Article" sheetId="1" r:id="rId1"/>
     <sheet name="Mots clés" sheetId="2" r:id="rId2"/>
     <sheet name="Prénom Nom Mail" sheetId="3" r:id="rId3"/>
-    <sheet name="Attribution par défault" sheetId="4" r:id="rId4"/>
+    <sheet name="Attribution par défaut" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Code et Article'!$E$1:$E$773</definedName>

</xml_diff>

<commit_message>
refactor: Move acronyms to the excel configuration file
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/mappings_attributions_for_tests.xlsx
+++ b/tests/integration/test_data/mappings_attributions_for_tests.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7BACA60-9038-5B49-BEE8-F2251AB66127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236BB80D-8312-3740-A4F0-54402370A91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Code et Article" sheetId="1" r:id="rId1"/>
     <sheet name="Mots clés" sheetId="2" r:id="rId2"/>
     <sheet name="Prénom Nom Mail" sheetId="3" r:id="rId3"/>
     <sheet name="Attribution par défaut" sheetId="4" r:id="rId4"/>
+    <sheet name="Acronymes" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Code et Article'!$E$1:$E$773</definedName>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="337">
   <si>
     <t>Bureau</t>
   </si>
@@ -257,6 +258,792 @@
   <si>
     <t>jmm@sante.gouv.fr</t>
   </si>
+  <si>
+    <t>Acronyme</t>
+  </si>
+  <si>
+    <t>Développement</t>
+  </si>
+  <si>
+    <t>AAH</t>
+  </si>
+  <si>
+    <t>allocation aux adultes handicapés</t>
+  </si>
+  <si>
+    <t>ACCRE</t>
+  </si>
+  <si>
+    <t>aide à la création ou à la reprise d'une entreprise</t>
+  </si>
+  <si>
+    <t>ACS</t>
+  </si>
+  <si>
+    <t>aide au paiement d'une complémentaire santé</t>
+  </si>
+  <si>
+    <t>AEEH</t>
+  </si>
+  <si>
+    <t>allocation d'éducation de l'enfant handicapé</t>
+  </si>
+  <si>
+    <t>AJPE</t>
+  </si>
+  <si>
+    <t>allocation journalière du proche aidant</t>
+  </si>
+  <si>
+    <t>AJPP</t>
+  </si>
+  <si>
+    <t>allocation journalière de présence parentale</t>
+  </si>
+  <si>
+    <t>ALD</t>
+  </si>
+  <si>
+    <t>affection longue durée</t>
+  </si>
+  <si>
+    <t>AME</t>
+  </si>
+  <si>
+    <t>aide médicale d'Etat</t>
+  </si>
+  <si>
+    <t>ANAP</t>
+  </si>
+  <si>
+    <t>agence nationale d'appui à la performance des établissements de santé et médico-sociaux</t>
+  </si>
+  <si>
+    <t>ANGDM</t>
+  </si>
+  <si>
+    <t>agence nationale de garantie des droits des mineurs</t>
+  </si>
+  <si>
+    <t>APL</t>
+  </si>
+  <si>
+    <t>aide personnalisée au logement</t>
+  </si>
+  <si>
+    <t>ASI</t>
+  </si>
+  <si>
+    <t>allocation supplémentaire d'invalidité</t>
+  </si>
+  <si>
+    <t>ASPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allocation de solidarité aux personnes âgées </t>
+  </si>
+  <si>
+    <t>AT/MP</t>
+  </si>
+  <si>
+    <t>acidents du travail - maladies professionnelles</t>
+  </si>
+  <si>
+    <t>ATIH</t>
+  </si>
+  <si>
+    <t>agence technique de l'information sur l'hospitalisation</t>
+  </si>
+  <si>
+    <t>AVA</t>
+  </si>
+  <si>
+    <t>assurance vieillesse des aidants</t>
+  </si>
+  <si>
+    <t>AVPF</t>
+  </si>
+  <si>
+    <t>assurance vieillesse des parents au foyer</t>
+  </si>
+  <si>
+    <t>C2S</t>
+  </si>
+  <si>
+    <t>complémentaire santé solidaire</t>
+  </si>
+  <si>
+    <t>C3S</t>
+  </si>
+  <si>
+    <t>contribution sociale de solidarité des sociétés</t>
+  </si>
+  <si>
+    <t>CADES</t>
+  </si>
+  <si>
+    <t>caisse d'amortissement de la dette sociale</t>
+  </si>
+  <si>
+    <t>CAF</t>
+  </si>
+  <si>
+    <t>caisse d'allocations familiales</t>
+  </si>
+  <si>
+    <t>CAMSP</t>
+  </si>
+  <si>
+    <t>centre d'action médico-sociale précoce</t>
+  </si>
+  <si>
+    <t>CANSSM</t>
+  </si>
+  <si>
+    <t>caisse autonome nationale de la sécurité sociale dans les mines</t>
+  </si>
+  <si>
+    <t>CARMF</t>
+  </si>
+  <si>
+    <t>caisse autonome de retraite des médecins de France</t>
+  </si>
+  <si>
+    <t>CARPIMKO</t>
+  </si>
+  <si>
+    <t>caisse autonome de retraite et de prévoyance des infirmiers, masseurs-kinésithérapeutes, orthophonistes, orthoptistes et pédicures-podologues</t>
+  </si>
+  <si>
+    <t>CARPV</t>
+  </si>
+  <si>
+    <t>caisse autonome de retraite et de prévoyance des vétérinaires</t>
+  </si>
+  <si>
+    <t>CAVAMAC</t>
+  </si>
+  <si>
+    <t>Caisse d’Allocation Vieillesse des Agents Généraux et des Mandataires non-salariés d’Assurance et de Capitalisation</t>
+  </si>
+  <si>
+    <t>CAVEC</t>
+  </si>
+  <si>
+    <t>Caisse d'assurance vieillesse des Experts-Comptables et des Commissaires aux comptes</t>
+  </si>
+  <si>
+    <t>CAVOM</t>
+  </si>
+  <si>
+    <t>caisse d'assurance vieillesse des officiers ministériels</t>
+  </si>
+  <si>
+    <t>CAVP</t>
+  </si>
+  <si>
+    <t>caisse d'assurance vieillesse des pharmaciens</t>
+  </si>
+  <si>
+    <t>CCAM</t>
+  </si>
+  <si>
+    <t>classification commune des actes médicaux</t>
+  </si>
+  <si>
+    <t>CCSF</t>
+  </si>
+  <si>
+    <t>commission des chefs des services financiers</t>
+  </si>
+  <si>
+    <t>CDAPH</t>
+  </si>
+  <si>
+    <t>commission des droits et de l'autonomie des personnes</t>
+  </si>
+  <si>
+    <t>CEPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comité économique des produits de santé </t>
+  </si>
+  <si>
+    <t>CER</t>
+  </si>
+  <si>
+    <t>cumul emploi retraite</t>
+  </si>
+  <si>
+    <t>CFE</t>
+  </si>
+  <si>
+    <t>caisse des français de l'étranger</t>
+  </si>
+  <si>
+    <t>CHM</t>
+  </si>
+  <si>
+    <t>centre hospitalier de Mayotte</t>
+  </si>
+  <si>
+    <t>CIAAF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collectif inter-associatif des aidants familiaux </t>
+  </si>
+  <si>
+    <t>CICE</t>
+  </si>
+  <si>
+    <t>crédit d'impôt compétitivité emploi</t>
+  </si>
+  <si>
+    <t>CIPAV</t>
+  </si>
+  <si>
+    <t>Caisse Interprofessionnelle de Prévoyance et d'Assurance Vieilless</t>
+  </si>
+  <si>
+    <t>CJUE</t>
+  </si>
+  <si>
+    <t>cour de justice de l'union européenne</t>
+  </si>
+  <si>
+    <t>CMU</t>
+  </si>
+  <si>
+    <t>couverture maladie universelle</t>
+  </si>
+  <si>
+    <t>CMU-C ACS</t>
+  </si>
+  <si>
+    <t>couverture maladie universelle complémentaire</t>
+  </si>
+  <si>
+    <t>CNAV</t>
+  </si>
+  <si>
+    <t>caisse nationale d'assurance vieillesse</t>
+  </si>
+  <si>
+    <t>CNG</t>
+  </si>
+  <si>
+    <t>centre national de gestion</t>
+  </si>
+  <si>
+    <t>CNH</t>
+  </si>
+  <si>
+    <t>commission nationale du handicap</t>
+  </si>
+  <si>
+    <t>CNSA</t>
+  </si>
+  <si>
+    <t>caisse nationale de solidarité pour l'autonomie</t>
+  </si>
+  <si>
+    <t>CNSE</t>
+  </si>
+  <si>
+    <t>centre national de soins à l'étranger</t>
+  </si>
+  <si>
+    <t>COR</t>
+  </si>
+  <si>
+    <t>conseil d'orientation des retraites</t>
+  </si>
+  <si>
+    <t>COREM</t>
+  </si>
+  <si>
+    <t>complément de retraite mutualiste</t>
+  </si>
+  <si>
+    <t>CPRN</t>
+  </si>
+  <si>
+    <t>caisse obligatoire de Prévoyance et de Retraite des Notaires libéraux</t>
+  </si>
+  <si>
+    <t>CRDS</t>
+  </si>
+  <si>
+    <t>contribution pour le remboursement de la dette sociale</t>
+  </si>
+  <si>
+    <t>CSA</t>
+  </si>
+  <si>
+    <t>contribution solidarité autonomie</t>
+  </si>
+  <si>
+    <t>CSG</t>
+  </si>
+  <si>
+    <t>contribution sociale généralisée</t>
+  </si>
+  <si>
+    <t>CSM</t>
+  </si>
+  <si>
+    <t>cotisation subsidiaire maladie</t>
+  </si>
+  <si>
+    <t>CSS</t>
+  </si>
+  <si>
+    <t>code de la sécurité sociale</t>
+  </si>
+  <si>
+    <t>CUMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coopératives d’utilisation de matériel agricole </t>
+  </si>
+  <si>
+    <t>CURPS</t>
+  </si>
+  <si>
+    <t>contribution aux unions régionales des professionnels de santé</t>
+  </si>
+  <si>
+    <t>EEE</t>
+  </si>
+  <si>
+    <t>espace économique européen</t>
+  </si>
+  <si>
+    <t>EHESP</t>
+  </si>
+  <si>
+    <t>école des hautes études en santé publique</t>
+  </si>
+  <si>
+    <t>EHPAD</t>
+  </si>
+  <si>
+    <t>établissement d'hébergement pour personnes âgées dépendantes</t>
+  </si>
+  <si>
+    <t>ESMS</t>
+  </si>
+  <si>
+    <t>établissement ou service médico-social</t>
+  </si>
+  <si>
+    <t>ETP</t>
+  </si>
+  <si>
+    <t>équivalent temps plein</t>
+  </si>
+  <si>
+    <t>FGTI</t>
+  </si>
+  <si>
+    <t>fonds de garantie des victimes de terrorisme et d'autres infractions</t>
+  </si>
+  <si>
+    <t>FHF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fédération hospitalière française </t>
+  </si>
+  <si>
+    <t>FIDES</t>
+  </si>
+  <si>
+    <t>facturation individuelle des établissements de santé</t>
+  </si>
+  <si>
+    <t>FIPU</t>
+  </si>
+  <si>
+    <t>fonds d'investissements dans la prévention de l'usure professionnelle</t>
+  </si>
+  <si>
+    <t>FIVA</t>
+  </si>
+  <si>
+    <t>fonds d'indemnisation des victimes de l'amiante</t>
+  </si>
+  <si>
+    <t>FMIS</t>
+  </si>
+  <si>
+    <t>fonds pour la modernisation et l'investissement en santé</t>
+  </si>
+  <si>
+    <t>FONPEL</t>
+  </si>
+  <si>
+    <t>fonds de pension des élus</t>
+  </si>
+  <si>
+    <t>FSV</t>
+  </si>
+  <si>
+    <t>fonds de solidarité vieillesse</t>
+  </si>
+  <si>
+    <t>GAEC</t>
+  </si>
+  <si>
+    <t>groupement agricole d'exploitation en commun </t>
+  </si>
+  <si>
+    <t>HAS</t>
+  </si>
+  <si>
+    <t>haute autorité de santé</t>
+  </si>
+  <si>
+    <t>HCAAM</t>
+  </si>
+  <si>
+    <t>haut conseil pour l'avenir de l'assurance maladie </t>
+  </si>
+  <si>
+    <t>HCFEA</t>
+  </si>
+  <si>
+    <t>haut conseil de la famille, de l’enfance et de l’âge</t>
+  </si>
+  <si>
+    <t>HCFiPS</t>
+  </si>
+  <si>
+    <t>haut conseil du financement de la protection sociale</t>
+  </si>
+  <si>
+    <t>IJ</t>
+  </si>
+  <si>
+    <t>indemnités journalières</t>
+  </si>
+  <si>
+    <t>IJSS</t>
+  </si>
+  <si>
+    <t>indemnités journalières de sécurité sociale</t>
+  </si>
+  <si>
+    <t>INSEE</t>
+  </si>
+  <si>
+    <t>institut national de la statistique et des études économiques</t>
+  </si>
+  <si>
+    <t>INSERM</t>
+  </si>
+  <si>
+    <t>institut national de la santé et de la recherche médicale</t>
+  </si>
+  <si>
+    <t>LAP</t>
+  </si>
+  <si>
+    <t>liste des actes et prescriptions</t>
+  </si>
+  <si>
+    <t>LFSS</t>
+  </si>
+  <si>
+    <t>loi de financement de la sécurité sociale</t>
+  </si>
+  <si>
+    <t>MCO</t>
+  </si>
+  <si>
+    <t>médecine, chirurgie, obstétrique</t>
+  </si>
+  <si>
+    <t>MDPH</t>
+  </si>
+  <si>
+    <t>maison départementale des personnes handicapées</t>
+  </si>
+  <si>
+    <t>MSA</t>
+  </si>
+  <si>
+    <t>mutualité sociale agricole</t>
+  </si>
+  <si>
+    <t>MTP</t>
+  </si>
+  <si>
+    <t>majoration pour tierce personne</t>
+  </si>
+  <si>
+    <t>NABM</t>
+  </si>
+  <si>
+    <t>nomenclature des actes de biologie médicale</t>
+  </si>
+  <si>
+    <t>NGAP</t>
+  </si>
+  <si>
+    <t>nomenclature générale des actes professionnels</t>
+  </si>
+  <si>
+    <t>OCDE</t>
+  </si>
+  <si>
+    <t>organisation de coopération et de développement économiques</t>
+  </si>
+  <si>
+    <t>OMS</t>
+  </si>
+  <si>
+    <t>organisation mondiale de la santé</t>
+  </si>
+  <si>
+    <t>ONDAM</t>
+  </si>
+  <si>
+    <t>objectif national de dépenses d'assurance maladie</t>
+  </si>
+  <si>
+    <t>OPTAM</t>
+  </si>
+  <si>
+    <t>option tarifaire maîtrisée</t>
+  </si>
+  <si>
+    <t>PADHUE</t>
+  </si>
+  <si>
+    <t>praticiens à diplôme hors UE</t>
+  </si>
+  <si>
+    <t>PAJE</t>
+  </si>
+  <si>
+    <t>prestation d'accueil du jeune enfant</t>
+  </si>
+  <si>
+    <t>PAMC</t>
+  </si>
+  <si>
+    <t>praticien et auxiliaire médical</t>
+  </si>
+  <si>
+    <t>PAP</t>
+  </si>
+  <si>
+    <t>projet annuel de performance</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>plafond annuel de la sécurité sociale</t>
+  </si>
+  <si>
+    <t>PEPS</t>
+  </si>
+  <si>
+    <t>paiement en équipe de professionnels de santé</t>
+  </si>
+  <si>
+    <t>PIB</t>
+  </si>
+  <si>
+    <t>produit intérieur brut</t>
+  </si>
+  <si>
+    <t>PLF</t>
+  </si>
+  <si>
+    <t>projet de loi de finances</t>
+  </si>
+  <si>
+    <t>PLFSS</t>
+  </si>
+  <si>
+    <t>projet de loi de financement de la sécurité sociale</t>
+  </si>
+  <si>
+    <t>PPL</t>
+  </si>
+  <si>
+    <t>proposition de loi</t>
+  </si>
+  <si>
+    <t>PPLO</t>
+  </si>
+  <si>
+    <t>proposition de loi organique</t>
+  </si>
+  <si>
+    <t>PPV</t>
+  </si>
+  <si>
+    <t>prime de partage de la valeur</t>
+  </si>
+  <si>
+    <t>PreParE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prestation partagée d’éducation de l’enfant </t>
+  </si>
+  <si>
+    <t>PREFON</t>
+  </si>
+  <si>
+    <t>caisse nationale de prévoyance de la fonction publique</t>
+  </si>
+  <si>
+    <t>PUMa / PUMA</t>
+  </si>
+  <si>
+    <t>protection universelle maladie</t>
+  </si>
+  <si>
+    <t>QVCT</t>
+  </si>
+  <si>
+    <t>qualité de vie et conditions de travail</t>
+  </si>
+  <si>
+    <t>RGD</t>
+  </si>
+  <si>
+    <t>réduction générale dégressive</t>
+  </si>
+  <si>
+    <t>RIHN</t>
+  </si>
+  <si>
+    <t>référentiel des actes innovants hors nomenclature</t>
+  </si>
+  <si>
+    <t>RSA</t>
+  </si>
+  <si>
+    <t>revenu de solidarité active</t>
+  </si>
+  <si>
+    <t>RSI</t>
+  </si>
+  <si>
+    <t>régime social des indépendants</t>
+  </si>
+  <si>
+    <t>RSPM</t>
+  </si>
+  <si>
+    <t>régime simplifié des professions médicales</t>
+  </si>
+  <si>
+    <t>SDREA</t>
+  </si>
+  <si>
+    <t>schéma directeur régional des exploitations agricoles</t>
+  </si>
+  <si>
+    <t>SAD</t>
+  </si>
+  <si>
+    <t>service autonomie à domicile</t>
+  </si>
+  <si>
+    <t>SMIC</t>
+  </si>
+  <si>
+    <t>salaire minimum interprofessionnel de croissance</t>
+  </si>
+  <si>
+    <t>SNGC</t>
+  </si>
+  <si>
+    <t>syndicat national de gérontologie clinique</t>
+  </si>
+  <si>
+    <t>SSIAD</t>
+  </si>
+  <si>
+    <t>services de soins infirmiers à domicile</t>
+  </si>
+  <si>
+    <t>T2A</t>
+  </si>
+  <si>
+    <t>tarification à l'activité</t>
+  </si>
+  <si>
+    <t>TND</t>
+  </si>
+  <si>
+    <t>troubles du neurodéveloppement</t>
+  </si>
+  <si>
+    <t>TO-DE</t>
+  </si>
+  <si>
+    <t>travailleurs occasionnels demandeurs d’emploi du secteur agricole</t>
+  </si>
+  <si>
+    <t>TPMR</t>
+  </si>
+  <si>
+    <t>transport de personnes à mobilité réduite</t>
+  </si>
+  <si>
+    <t>TPT</t>
+  </si>
+  <si>
+    <t>temps partiel pour raison thérapeutique</t>
+  </si>
+  <si>
+    <t>TSA</t>
+  </si>
+  <si>
+    <t>taxe de solidarité additionnelle</t>
+  </si>
+  <si>
+    <t>TVA</t>
+  </si>
+  <si>
+    <t>taxe sur la valeur ajoutée</t>
+  </si>
+  <si>
+    <t>UE</t>
+  </si>
+  <si>
+    <t>union européenne</t>
+  </si>
+  <si>
+    <t>UNAF</t>
+  </si>
+  <si>
+    <t>union nationale des associations familiales</t>
+  </si>
+  <si>
+    <t>URPS</t>
+  </si>
+  <si>
+    <t>union régionale des professionnels de santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USLD </t>
+  </si>
+  <si>
+    <t>unités de soins de longue durée</t>
+  </si>
+  <si>
+    <t>VPH</t>
+  </si>
+  <si>
+    <t>véhicules pour personne en situation de handicap</t>
+  </si>
 </sst>
 </file>
 
@@ -266,7 +1053,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-m\-d"/>
     <numFmt numFmtId="165" formatCode="yyyy\-m"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -344,8 +1131,21 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -356,6 +1156,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8EA9DB"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -378,7 +1184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -441,6 +1247,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32245,4 +33056,1066 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E07DC06-BE6F-E74C-AC13-6CDBAAED5E7C}">
+  <dimension ref="A1:B131"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="104.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B27" s="27" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="28" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="B33" s="27" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="B39" s="27" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="B41" s="27" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="B42" s="27" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="B43" s="27" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B44" s="27" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="B45" s="27" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B46" s="27" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="27" t="s">
+        <v>167</v>
+      </c>
+      <c r="B47" s="27" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="B48" s="27" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="B49" s="27" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B50" s="27" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="B51" s="27" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="B52" s="27" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="B53" s="27" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="B54" s="27" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="27" t="s">
+        <v>183</v>
+      </c>
+      <c r="B55" s="27" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="B56" s="27" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="27" t="s">
+        <v>187</v>
+      </c>
+      <c r="B57" s="27" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="27" t="s">
+        <v>189</v>
+      </c>
+      <c r="B58" s="27" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="27" t="s">
+        <v>191</v>
+      </c>
+      <c r="B59" s="27" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="B60" s="27" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="B61" s="27" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="27" t="s">
+        <v>197</v>
+      </c>
+      <c r="B62" s="27" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="27" t="s">
+        <v>199</v>
+      </c>
+      <c r="B63" s="27" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="27" t="s">
+        <v>201</v>
+      </c>
+      <c r="B64" s="27" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="B65" s="27" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="27" t="s">
+        <v>205</v>
+      </c>
+      <c r="B66" s="27" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="B67" s="27" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="B68" s="27" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="B69" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="B70" s="27" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="B71" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="B72" s="27" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="27" t="s">
+        <v>219</v>
+      </c>
+      <c r="B73" s="27" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="B74" s="27" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="B75" s="27" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="B76" s="27" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="27" t="s">
+        <v>227</v>
+      </c>
+      <c r="B77" s="27" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="27" t="s">
+        <v>229</v>
+      </c>
+      <c r="B78" s="27" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="27" t="s">
+        <v>231</v>
+      </c>
+      <c r="B79" s="27" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="B80" s="27" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="27" t="s">
+        <v>235</v>
+      </c>
+      <c r="B81" s="27" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="27" t="s">
+        <v>237</v>
+      </c>
+      <c r="B82" s="27" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="27" t="s">
+        <v>239</v>
+      </c>
+      <c r="B83" s="27" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="B84" s="27" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="B85" s="27" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="27" t="s">
+        <v>245</v>
+      </c>
+      <c r="B86" s="27" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="B87" s="27" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="B88" s="27" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="B89" s="27" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="B90" s="27" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="B91" s="27" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="B92" s="27" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="27" t="s">
+        <v>259</v>
+      </c>
+      <c r="B93" s="27" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="27" t="s">
+        <v>261</v>
+      </c>
+      <c r="B94" s="27" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="27" t="s">
+        <v>263</v>
+      </c>
+      <c r="B95" s="27" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="27" t="s">
+        <v>265</v>
+      </c>
+      <c r="B96" s="27" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="27" t="s">
+        <v>267</v>
+      </c>
+      <c r="B97" s="27" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="27" t="s">
+        <v>269</v>
+      </c>
+      <c r="B98" s="27" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="27" t="s">
+        <v>271</v>
+      </c>
+      <c r="B99" s="27" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="B100" s="27" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="27" t="s">
+        <v>275</v>
+      </c>
+      <c r="B101" s="27" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="27" t="s">
+        <v>277</v>
+      </c>
+      <c r="B102" s="27" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="B103" s="27" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="B104" s="27" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="B105" s="27" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" s="27" t="s">
+        <v>285</v>
+      </c>
+      <c r="B106" s="27" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="27" t="s">
+        <v>287</v>
+      </c>
+      <c r="B107" s="27" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" s="27" t="s">
+        <v>289</v>
+      </c>
+      <c r="B108" s="27" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="27" t="s">
+        <v>291</v>
+      </c>
+      <c r="B109" s="27" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" s="27" t="s">
+        <v>293</v>
+      </c>
+      <c r="B110" s="27" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="B111" s="27" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" s="27" t="s">
+        <v>297</v>
+      </c>
+      <c r="B112" s="27" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="B113" s="27" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="27" t="s">
+        <v>301</v>
+      </c>
+      <c r="B114" s="27" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="27" t="s">
+        <v>303</v>
+      </c>
+      <c r="B115" s="27" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="B116" s="27" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="B117" s="27" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="27" t="s">
+        <v>309</v>
+      </c>
+      <c r="B118" s="27" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="B119" s="27" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="27" t="s">
+        <v>313</v>
+      </c>
+      <c r="B120" s="27" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="27" t="s">
+        <v>315</v>
+      </c>
+      <c r="B121" s="27" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="27" t="s">
+        <v>317</v>
+      </c>
+      <c r="B122" s="27" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="27" t="s">
+        <v>319</v>
+      </c>
+      <c r="B123" s="27" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" s="27" t="s">
+        <v>321</v>
+      </c>
+      <c r="B124" s="27" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" s="27" t="s">
+        <v>323</v>
+      </c>
+      <c r="B125" s="27" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" s="27" t="s">
+        <v>325</v>
+      </c>
+      <c r="B126" s="27" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" s="27" t="s">
+        <v>327</v>
+      </c>
+      <c r="B127" s="27" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" s="27" t="s">
+        <v>329</v>
+      </c>
+      <c r="B128" s="27" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" s="27" t="s">
+        <v>331</v>
+      </c>
+      <c r="B129" s="27" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" s="27" t="s">
+        <v>333</v>
+      </c>
+      <c r="B130" s="27" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" s="27" t="s">
+        <v>335</v>
+      </c>
+      <c r="B131" s="27" t="s">
+        <v>336</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat (attribution): Add "Entité Pilote" to attribution
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/mappings_attributions_for_tests.xlsx
+++ b/tests/integration/test_data/mappings_attributions_for_tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236BB80D-8312-3740-A4F0-54402370A91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE632D3-FA68-344C-AB70-2A63035DBCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Code et Article" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="342">
   <si>
     <t>Bureau</t>
   </si>
@@ -1044,6 +1044,21 @@
   <si>
     <t>véhicules pour personne en situation de handicap</t>
   </si>
+  <si>
+    <t>Entité pilote</t>
+  </si>
+  <si>
+    <t>MABC</t>
+  </si>
+  <si>
+    <t>NABC</t>
+  </si>
+  <si>
+    <t>JABC</t>
+  </si>
+  <si>
+    <t>EABC</t>
+  </si>
 </sst>
 </file>
 
@@ -30940,7 +30955,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B1000"/>
+  <dimension ref="A1:C999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.1640625" customWidth="1"/>
@@ -30948,92 +30963,112 @@
     <col min="3" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" customHeight="1">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1">
+      <c r="C1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1">
       <c r="A2" s="21" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="22" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1">
+      <c r="C2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1">
       <c r="A3" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="22" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1">
+      <c r="C3" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" customHeight="1">
       <c r="A4" s="21" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="22" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1">
+      <c r="C4" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" customHeight="1">
       <c r="A5" s="21" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="22" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1">
+      <c r="C5" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1">
       <c r="A6" s="13" t="s">
         <v>39</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A7" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A8" s="17" t="s">
+      <c r="C6" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A7" s="17" t="s">
         <v>70</v>
       </c>
+      <c r="B7" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A8" s="23" t="s">
+        <v>72</v>
+      </c>
       <c r="B8" s="22" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A9" s="23" t="s">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A9" s="24" t="s">
+        <v>60</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A10" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="22" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="12" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="13" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="14" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="16" spans="1:2" ht="15.75" customHeight="1"/>
+      <c r="C9" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="11" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="12" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="13" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="14" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="15" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="16" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -32017,16 +32052,15 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
     <hyperlink ref="B5" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
-    <hyperlink ref="B8" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
-    <hyperlink ref="B9" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
-    <hyperlink ref="B10" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="B7" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="B9" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
fix(attribution): Bug with punctuation and keyword matching
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/mappings_attributions_for_tests.xlsx
+++ b/tests/integration/test_data/mappings_attributions_for_tests.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE632D3-FA68-344C-AB70-2A63035DBCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7DB789-95B7-724C-A485-307EEAA8B036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="346">
   <si>
     <t>Bureau</t>
   </si>
@@ -1045,9 +1045,6 @@
     <t>véhicules pour personne en situation de handicap</t>
   </si>
   <si>
-    <t>Entité pilote</t>
-  </si>
-  <si>
     <t>MABC</t>
   </si>
   <si>
@@ -1058,6 +1055,21 @@
   </si>
   <si>
     <t>EABC</t>
+  </si>
+  <si>
+    <t>Entité Pilote</t>
+  </si>
+  <si>
+    <t>Charlotte Legresy</t>
+  </si>
+  <si>
+    <t>établissement français du sang</t>
+  </si>
+  <si>
+    <t>charlotte.legresy@sante.gouv.fr</t>
+  </si>
+  <si>
+    <t>CABC</t>
   </si>
 </sst>
 </file>
@@ -1068,7 +1080,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-m\-d"/>
     <numFmt numFmtId="165" formatCode="yyyy\-m"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1124,21 +1136,9 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1157,6 +1157,26 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1196,10 +1216,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1255,20 +1276,31 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3200,8 +3232,12 @@
       <c r="Z9" s="13"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A10" s="16"/>
-      <c r="B10" s="15"/>
+      <c r="A10" s="26" t="s">
+        <v>343</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>342</v>
+      </c>
       <c r="C10" s="15"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
@@ -30964,105 +31000,115 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="28" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A2" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A2" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="3" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A3" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A4" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="29" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A3" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="5" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A5" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A6" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A7" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A8" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="29" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A4" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="9" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A9" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="29" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A5" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A6" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A7" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="C7" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A8" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A9" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="10" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A10" s="29" t="s">
+        <v>342</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>344</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>345</v>
+      </c>
+    </row>
     <row r="11" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="12" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="13" spans="1:3" ht="15.75" customHeight="1"/>
@@ -32061,6 +32107,7 @@
     <hyperlink ref="B7" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
     <hyperlink ref="B8" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
     <hyperlink ref="B9" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="B10" r:id="rId8" xr:uid="{CFDE7F7F-C31D-A24F-BFF6-DB7DD59714EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -32077,17 +32124,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="22" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="21" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1">
-      <c r="A3" s="23"/>
+      <c r="A3" s="21"/>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1"/>
     <row r="5" spans="1:1" ht="15.75" customHeight="1"/>
@@ -33102,1050 +33149,1050 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="23" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="24" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="24" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="24" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="24" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="24" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="24" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="24" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="24" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="24" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="24" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="24" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="24" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="24" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="24" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="24" t="s">
         <v>105</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="24" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="24" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="24" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="27" t="s">
+      <c r="A19" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="24" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="24" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="24" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="27" t="s">
+      <c r="A22" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="B22" s="27" t="s">
+      <c r="B22" s="24" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="27" t="s">
+      <c r="A23" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="24" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="B24" s="27" t="s">
+      <c r="B24" s="24" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="B25" s="27" t="s">
+      <c r="B25" s="24" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="24" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="24" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="B28" s="27" t="s">
+      <c r="B28" s="24" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="28" t="s">
+      <c r="A29" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="B29" s="27" t="s">
+      <c r="B29" s="24" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="B30" s="27" t="s">
+      <c r="B30" s="24" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="24" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="24" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="24" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="27" t="s">
+      <c r="A34" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="27" t="s">
+      <c r="B34" s="24" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="B35" s="27" t="s">
+      <c r="B35" s="24" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="27" t="s">
+      <c r="A36" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="B36" s="27" t="s">
+      <c r="B36" s="24" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="27" t="s">
+      <c r="A37" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="B37" s="27" t="s">
+      <c r="B37" s="24" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="27" t="s">
+      <c r="A38" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="B38" s="27" t="s">
+      <c r="B38" s="24" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="27" t="s">
+      <c r="A39" s="24" t="s">
         <v>151</v>
       </c>
-      <c r="B39" s="27" t="s">
+      <c r="B39" s="24" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="27" t="s">
+      <c r="A40" s="24" t="s">
         <v>153</v>
       </c>
-      <c r="B40" s="27" t="s">
+      <c r="B40" s="24" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="28" t="s">
+      <c r="A41" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="B41" s="27" t="s">
+      <c r="B41" s="24" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="27" t="s">
+      <c r="A42" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="B42" s="27" t="s">
+      <c r="B42" s="24" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="27" t="s">
+      <c r="A43" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="B43" s="27" t="s">
+      <c r="B43" s="24" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="27" t="s">
+      <c r="A44" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="B44" s="27" t="s">
+      <c r="B44" s="24" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="27" t="s">
+      <c r="A45" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="B45" s="27" t="s">
+      <c r="B45" s="24" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="27" t="s">
+      <c r="A46" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="B46" s="27" t="s">
+      <c r="B46" s="24" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="27" t="s">
+      <c r="A47" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="B47" s="27" t="s">
+      <c r="B47" s="24" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="27" t="s">
+      <c r="A48" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B48" s="27" t="s">
+      <c r="B48" s="24" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="27" t="s">
+      <c r="A49" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="B49" s="27" t="s">
+      <c r="B49" s="24" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="50" spans="1:2">
-      <c r="A50" s="27" t="s">
+      <c r="A50" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="B50" s="27" t="s">
+      <c r="B50" s="24" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="51" spans="1:2">
-      <c r="A51" s="27" t="s">
+      <c r="A51" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="B51" s="27" t="s">
+      <c r="B51" s="24" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="52" spans="1:2">
-      <c r="A52" s="28" t="s">
+      <c r="A52" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="B52" s="27" t="s">
+      <c r="B52" s="24" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="53" spans="1:2">
-      <c r="A53" s="27" t="s">
+      <c r="A53" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="B53" s="27" t="s">
+      <c r="B53" s="24" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="54" spans="1:2">
-      <c r="A54" s="27" t="s">
+      <c r="A54" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="B54" s="27" t="s">
+      <c r="B54" s="24" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="55" spans="1:2">
-      <c r="A55" s="27" t="s">
+      <c r="A55" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="B55" s="27" t="s">
+      <c r="B55" s="24" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="56" spans="1:2">
-      <c r="A56" s="27" t="s">
+      <c r="A56" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="B56" s="27" t="s">
+      <c r="B56" s="24" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="57" spans="1:2">
-      <c r="A57" s="27" t="s">
+      <c r="A57" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="B57" s="27" t="s">
+      <c r="B57" s="24" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="58" spans="1:2">
-      <c r="A58" s="27" t="s">
+      <c r="A58" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="B58" s="27" t="s">
+      <c r="B58" s="24" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="59" spans="1:2">
-      <c r="A59" s="27" t="s">
+      <c r="A59" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="B59" s="27" t="s">
+      <c r="B59" s="24" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="60" spans="1:2">
-      <c r="A60" s="27" t="s">
+      <c r="A60" s="24" t="s">
         <v>193</v>
       </c>
-      <c r="B60" s="27" t="s">
+      <c r="B60" s="24" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="61" spans="1:2">
-      <c r="A61" s="27" t="s">
+      <c r="A61" s="24" t="s">
         <v>195</v>
       </c>
-      <c r="B61" s="27" t="s">
+      <c r="B61" s="24" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="62" spans="1:2">
-      <c r="A62" s="27" t="s">
+      <c r="A62" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="B62" s="27" t="s">
+      <c r="B62" s="24" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="63" spans="1:2">
-      <c r="A63" s="27" t="s">
+      <c r="A63" s="24" t="s">
         <v>199</v>
       </c>
-      <c r="B63" s="27" t="s">
+      <c r="B63" s="24" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:2">
-      <c r="A64" s="27" t="s">
+      <c r="A64" s="24" t="s">
         <v>201</v>
       </c>
-      <c r="B64" s="27" t="s">
+      <c r="B64" s="24" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="65" spans="1:2">
-      <c r="A65" s="27" t="s">
+      <c r="A65" s="24" t="s">
         <v>203</v>
       </c>
-      <c r="B65" s="27" t="s">
+      <c r="B65" s="24" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="66" spans="1:2">
-      <c r="A66" s="27" t="s">
+      <c r="A66" s="24" t="s">
         <v>205</v>
       </c>
-      <c r="B66" s="27" t="s">
+      <c r="B66" s="24" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="67" spans="1:2">
-      <c r="A67" s="27" t="s">
+      <c r="A67" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="B67" s="27" t="s">
+      <c r="B67" s="24" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="68" spans="1:2">
-      <c r="A68" s="27" t="s">
+      <c r="A68" s="24" t="s">
         <v>209</v>
       </c>
-      <c r="B68" s="27" t="s">
+      <c r="B68" s="24" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="69" spans="1:2">
-      <c r="A69" s="27" t="s">
+      <c r="A69" s="24" t="s">
         <v>211</v>
       </c>
-      <c r="B69" s="27" t="s">
+      <c r="B69" s="24" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="70" spans="1:2">
-      <c r="A70" s="27" t="s">
+      <c r="A70" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="B70" s="27" t="s">
+      <c r="B70" s="24" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="71" spans="1:2">
-      <c r="A71" s="27" t="s">
+      <c r="A71" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="B71" s="27" t="s">
+      <c r="B71" s="24" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="72" spans="1:2">
-      <c r="A72" s="27" t="s">
+      <c r="A72" s="24" t="s">
         <v>217</v>
       </c>
-      <c r="B72" s="27" t="s">
+      <c r="B72" s="24" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="73" spans="1:2">
-      <c r="A73" s="27" t="s">
+      <c r="A73" s="24" t="s">
         <v>219</v>
       </c>
-      <c r="B73" s="27" t="s">
+      <c r="B73" s="24" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="74" spans="1:2">
-      <c r="A74" s="27" t="s">
+      <c r="A74" s="24" t="s">
         <v>221</v>
       </c>
-      <c r="B74" s="27" t="s">
+      <c r="B74" s="24" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="75" spans="1:2">
-      <c r="A75" s="27" t="s">
+      <c r="A75" s="24" t="s">
         <v>223</v>
       </c>
-      <c r="B75" s="27" t="s">
+      <c r="B75" s="24" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="76" spans="1:2">
-      <c r="A76" s="27" t="s">
+      <c r="A76" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="B76" s="27" t="s">
+      <c r="B76" s="24" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="77" spans="1:2">
-      <c r="A77" s="27" t="s">
+      <c r="A77" s="24" t="s">
         <v>227</v>
       </c>
-      <c r="B77" s="27" t="s">
+      <c r="B77" s="24" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="78" spans="1:2">
-      <c r="A78" s="27" t="s">
+      <c r="A78" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="B78" s="27" t="s">
+      <c r="B78" s="24" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="79" spans="1:2">
-      <c r="A79" s="27" t="s">
+      <c r="A79" s="24" t="s">
         <v>231</v>
       </c>
-      <c r="B79" s="27" t="s">
+      <c r="B79" s="24" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="80" spans="1:2">
-      <c r="A80" s="27" t="s">
+      <c r="A80" s="24" t="s">
         <v>233</v>
       </c>
-      <c r="B80" s="27" t="s">
+      <c r="B80" s="24" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="81" spans="1:2">
-      <c r="A81" s="27" t="s">
+      <c r="A81" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="B81" s="27" t="s">
+      <c r="B81" s="24" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="82" spans="1:2">
-      <c r="A82" s="27" t="s">
+      <c r="A82" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="B82" s="27" t="s">
+      <c r="B82" s="24" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="83" spans="1:2">
-      <c r="A83" s="27" t="s">
+      <c r="A83" s="24" t="s">
         <v>239</v>
       </c>
-      <c r="B83" s="27" t="s">
+      <c r="B83" s="24" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="84" spans="1:2">
-      <c r="A84" s="27" t="s">
+      <c r="A84" s="24" t="s">
         <v>241</v>
       </c>
-      <c r="B84" s="27" t="s">
+      <c r="B84" s="24" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="85" spans="1:2">
-      <c r="A85" s="27" t="s">
+      <c r="A85" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="B85" s="27" t="s">
+      <c r="B85" s="24" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="86" spans="1:2">
-      <c r="A86" s="27" t="s">
+      <c r="A86" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="B86" s="27" t="s">
+      <c r="B86" s="24" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="87" spans="1:2">
-      <c r="A87" s="27" t="s">
+      <c r="A87" s="24" t="s">
         <v>247</v>
       </c>
-      <c r="B87" s="27" t="s">
+      <c r="B87" s="24" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="88" spans="1:2">
-      <c r="A88" s="27" t="s">
+      <c r="A88" s="24" t="s">
         <v>249</v>
       </c>
-      <c r="B88" s="27" t="s">
+      <c r="B88" s="24" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="89" spans="1:2">
-      <c r="A89" s="27" t="s">
+      <c r="A89" s="24" t="s">
         <v>251</v>
       </c>
-      <c r="B89" s="27" t="s">
+      <c r="B89" s="24" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="90" spans="1:2">
-      <c r="A90" s="27" t="s">
+      <c r="A90" s="24" t="s">
         <v>253</v>
       </c>
-      <c r="B90" s="27" t="s">
+      <c r="B90" s="24" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="91" spans="1:2">
-      <c r="A91" s="27" t="s">
+      <c r="A91" s="24" t="s">
         <v>255</v>
       </c>
-      <c r="B91" s="27" t="s">
+      <c r="B91" s="24" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="92" spans="1:2">
-      <c r="A92" s="27" t="s">
+      <c r="A92" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="B92" s="27" t="s">
+      <c r="B92" s="24" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="93" spans="1:2">
-      <c r="A93" s="27" t="s">
+      <c r="A93" s="24" t="s">
         <v>259</v>
       </c>
-      <c r="B93" s="27" t="s">
+      <c r="B93" s="24" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="94" spans="1:2">
-      <c r="A94" s="27" t="s">
+      <c r="A94" s="24" t="s">
         <v>261</v>
       </c>
-      <c r="B94" s="27" t="s">
+      <c r="B94" s="24" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="95" spans="1:2">
-      <c r="A95" s="27" t="s">
+      <c r="A95" s="24" t="s">
         <v>263</v>
       </c>
-      <c r="B95" s="27" t="s">
+      <c r="B95" s="24" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="96" spans="1:2">
-      <c r="A96" s="27" t="s">
+      <c r="A96" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="B96" s="27" t="s">
+      <c r="B96" s="24" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="97" spans="1:2">
-      <c r="A97" s="27" t="s">
+      <c r="A97" s="24" t="s">
         <v>267</v>
       </c>
-      <c r="B97" s="27" t="s">
+      <c r="B97" s="24" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="98" spans="1:2">
-      <c r="A98" s="27" t="s">
+      <c r="A98" s="24" t="s">
         <v>269</v>
       </c>
-      <c r="B98" s="27" t="s">
+      <c r="B98" s="24" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="99" spans="1:2">
-      <c r="A99" s="27" t="s">
+      <c r="A99" s="24" t="s">
         <v>271</v>
       </c>
-      <c r="B99" s="27" t="s">
+      <c r="B99" s="24" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="100" spans="1:2">
-      <c r="A100" s="27" t="s">
+      <c r="A100" s="24" t="s">
         <v>273</v>
       </c>
-      <c r="B100" s="27" t="s">
+      <c r="B100" s="24" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="101" spans="1:2">
-      <c r="A101" s="27" t="s">
+      <c r="A101" s="24" t="s">
         <v>275</v>
       </c>
-      <c r="B101" s="27" t="s">
+      <c r="B101" s="24" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="102" spans="1:2">
-      <c r="A102" s="27" t="s">
+      <c r="A102" s="24" t="s">
         <v>277</v>
       </c>
-      <c r="B102" s="27" t="s">
+      <c r="B102" s="24" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="103" spans="1:2">
-      <c r="A103" s="27" t="s">
+      <c r="A103" s="24" t="s">
         <v>279</v>
       </c>
-      <c r="B103" s="27" t="s">
+      <c r="B103" s="24" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="104" spans="1:2">
-      <c r="A104" s="27" t="s">
+      <c r="A104" s="24" t="s">
         <v>281</v>
       </c>
-      <c r="B104" s="27" t="s">
+      <c r="B104" s="24" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="105" spans="1:2">
-      <c r="A105" s="27" t="s">
+      <c r="A105" s="24" t="s">
         <v>283</v>
       </c>
-      <c r="B105" s="27" t="s">
+      <c r="B105" s="24" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="106" spans="1:2">
-      <c r="A106" s="27" t="s">
+      <c r="A106" s="24" t="s">
         <v>285</v>
       </c>
-      <c r="B106" s="27" t="s">
+      <c r="B106" s="24" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="107" spans="1:2">
-      <c r="A107" s="27" t="s">
+      <c r="A107" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="B107" s="27" t="s">
+      <c r="B107" s="24" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="108" spans="1:2">
-      <c r="A108" s="27" t="s">
+      <c r="A108" s="24" t="s">
         <v>289</v>
       </c>
-      <c r="B108" s="27" t="s">
+      <c r="B108" s="24" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="109" spans="1:2">
-      <c r="A109" s="27" t="s">
+      <c r="A109" s="24" t="s">
         <v>291</v>
       </c>
-      <c r="B109" s="27" t="s">
+      <c r="B109" s="24" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="110" spans="1:2">
-      <c r="A110" s="27" t="s">
+      <c r="A110" s="24" t="s">
         <v>293</v>
       </c>
-      <c r="B110" s="27" t="s">
+      <c r="B110" s="24" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="111" spans="1:2">
-      <c r="A111" s="27" t="s">
+      <c r="A111" s="24" t="s">
         <v>295</v>
       </c>
-      <c r="B111" s="27" t="s">
+      <c r="B111" s="24" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="112" spans="1:2">
-      <c r="A112" s="27" t="s">
+      <c r="A112" s="24" t="s">
         <v>297</v>
       </c>
-      <c r="B112" s="27" t="s">
+      <c r="B112" s="24" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="113" spans="1:2">
-      <c r="A113" s="27" t="s">
+      <c r="A113" s="24" t="s">
         <v>299</v>
       </c>
-      <c r="B113" s="27" t="s">
+      <c r="B113" s="24" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="114" spans="1:2">
-      <c r="A114" s="27" t="s">
+      <c r="A114" s="24" t="s">
         <v>301</v>
       </c>
-      <c r="B114" s="27" t="s">
+      <c r="B114" s="24" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="115" spans="1:2">
-      <c r="A115" s="27" t="s">
+      <c r="A115" s="24" t="s">
         <v>303</v>
       </c>
-      <c r="B115" s="27" t="s">
+      <c r="B115" s="24" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="116" spans="1:2">
-      <c r="A116" s="27" t="s">
+      <c r="A116" s="24" t="s">
         <v>305</v>
       </c>
-      <c r="B116" s="27" t="s">
+      <c r="B116" s="24" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="117" spans="1:2">
-      <c r="A117" s="27" t="s">
+      <c r="A117" s="24" t="s">
         <v>307</v>
       </c>
-      <c r="B117" s="27" t="s">
+      <c r="B117" s="24" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="118" spans="1:2">
-      <c r="A118" s="27" t="s">
+      <c r="A118" s="24" t="s">
         <v>309</v>
       </c>
-      <c r="B118" s="27" t="s">
+      <c r="B118" s="24" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="119" spans="1:2">
-      <c r="A119" s="27" t="s">
+      <c r="A119" s="24" t="s">
         <v>311</v>
       </c>
-      <c r="B119" s="27" t="s">
+      <c r="B119" s="24" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="120" spans="1:2">
-      <c r="A120" s="27" t="s">
+      <c r="A120" s="24" t="s">
         <v>313</v>
       </c>
-      <c r="B120" s="27" t="s">
+      <c r="B120" s="24" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="121" spans="1:2">
-      <c r="A121" s="27" t="s">
+      <c r="A121" s="24" t="s">
         <v>315</v>
       </c>
-      <c r="B121" s="27" t="s">
+      <c r="B121" s="24" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="122" spans="1:2">
-      <c r="A122" s="27" t="s">
+      <c r="A122" s="24" t="s">
         <v>317</v>
       </c>
-      <c r="B122" s="27" t="s">
+      <c r="B122" s="24" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="123" spans="1:2">
-      <c r="A123" s="27" t="s">
+      <c r="A123" s="24" t="s">
         <v>319</v>
       </c>
-      <c r="B123" s="27" t="s">
+      <c r="B123" s="24" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="124" spans="1:2">
-      <c r="A124" s="27" t="s">
+      <c r="A124" s="24" t="s">
         <v>321</v>
       </c>
-      <c r="B124" s="27" t="s">
+      <c r="B124" s="24" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="125" spans="1:2">
-      <c r="A125" s="27" t="s">
+      <c r="A125" s="24" t="s">
         <v>323</v>
       </c>
-      <c r="B125" s="27" t="s">
+      <c r="B125" s="24" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="126" spans="1:2">
-      <c r="A126" s="27" t="s">
+      <c r="A126" s="24" t="s">
         <v>325</v>
       </c>
-      <c r="B126" s="27" t="s">
+      <c r="B126" s="24" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="127" spans="1:2">
-      <c r="A127" s="27" t="s">
+      <c r="A127" s="24" t="s">
         <v>327</v>
       </c>
-      <c r="B127" s="27" t="s">
+      <c r="B127" s="24" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="128" spans="1:2">
-      <c r="A128" s="27" t="s">
+      <c r="A128" s="24" t="s">
         <v>329</v>
       </c>
-      <c r="B128" s="27" t="s">
+      <c r="B128" s="24" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="129" spans="1:2">
-      <c r="A129" s="27" t="s">
+      <c r="A129" s="24" t="s">
         <v>331</v>
       </c>
-      <c r="B129" s="27" t="s">
+      <c r="B129" s="24" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="130" spans="1:2">
-      <c r="A130" s="27" t="s">
+      <c r="A130" s="24" t="s">
         <v>333</v>
       </c>
-      <c r="B130" s="27" t="s">
+      <c r="B130" s="24" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="131" spans="1:2">
-      <c r="A131" s="27" t="s">
+      <c r="A131" s="24" t="s">
         <v>335</v>
       </c>
-      <c r="B131" s="27" t="s">
+      <c r="B131" s="24" t="s">
         <v>336</v>
       </c>
     </row>

</xml_diff>